<commit_message>
feat: connect UI snapshot and implement changeover protection
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Ui/UI_Board_Validation.xlsx
+++ b/Firmware/Modules/Ui/UI_Board_Validation.xlsx
@@ -494,7 +494,7 @@
     <tabColor rgb="70AD47"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S44"/>
+  <dimension ref="A1:S50"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -4207,24 +4207,456 @@
         </is>
       </c>
     </row>
+    <row r="45" ht="58" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI-034</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measurement</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">بالا</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پس از Init یا شکست ADC، snapshot.valid=false</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0V / 0V</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">همه LED و بوق خاموش؛ آلارم باتری false</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">safe-off و بدون BatteryRun</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="58" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI-035</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measurement</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">بالا</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snapshot.valid=true؛ input_present=false؛ vbat=28000mV</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0V / 28V</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BatteryRun؛ آلارم کم‌باتری false</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ورودی قطع و باتری فول معتبر</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="58" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI-036</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">InputOk</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">بالا</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snapshot.valid=true؛ input_present=true؛ vbat=28000mV</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24V / 28V</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">سبز دائم؛ زرد/قرمز/بوق خاموش</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">منبع متصل و باتری فول</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M47" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N47" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="58" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI-037</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Charging</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">متوسط</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snapshot.valid=true؛ input_present=true؛ vbat=25000mV</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24V / 25V</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">سبز دائم؛ زرد چشمک؛ بوق خاموش</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">باتری در حال شارژ</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M48" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N48" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="58" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI-038</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OverVoltage</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">بالا</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snapshot.valid=true؛ v_in&gt;28000mV</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29V / 25V</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">قرمز چشمک و بوق طبق جدول</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">آستانه از v_in معتبر</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M49" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N49" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="58" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI-039</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LowBattery flag</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">بالا</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snapshot.valid=true؛ input_present=false؛ vbat&lt;21000mV</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0V / 20.9V</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low Battery Alarm فعال؛ UiBatteryAlarmIssued=true</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">فلگ سطحی برای مصرف Changeover</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:S44"/>
+  <autoFilter ref="A4:S50"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="C5:C44">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="C5:C50">
       <formula1>بالا,متوسط,پایین</formula1>
       <promptTitle>اولویت</promptTitle>
       <prompt>اولویت تست را انتخاب کن.</prompt>
       <errorTitle>مقدار نامعتبر</errorTitle>
       <error>یکی از گزینه‌های فهرست را انتخاب کن.</error>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="N5:N44">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="N5:N50">
       <formula1>در انتظار,قبول,رد,مسدود,نیاز به تکرار</formula1>
       <promptTitle>وضعیت تست</promptTitle>
       <prompt>بعد از مشاهدهٔ نتیجه انتخاب کن.</prompt>
       <errorTitle>مقدار نامعتبر</errorTitle>
       <error>وضعیت را از فهرست انتخاب کن.</error>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="S5:S44">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorStyle="stop" sqref="S5:S50">
       <formula1>در انتظار,تأیید شد,تأیید نشد,نیاز به بررسی</formula1>
       <promptTitle>تأیید تست</promptTitle>
       <prompt>پس از ثبت نتیجه تصمیم بگیر.</prompt>
@@ -4232,32 +4664,32 @@
       <error>وضعیت تأیید را از فهرست انتخاب کن.</error>
     </dataValidation>
   </dataValidations>
-  <conditionalFormatting sqref="N5:N44">
+  <conditionalFormatting sqref="N5:N50">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>N5="قبول"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N44">
+  <conditionalFormatting sqref="N5:N50">
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>N5="رد"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N44">
+  <conditionalFormatting sqref="N5:N50">
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>N5="مسدود"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N44">
+  <conditionalFormatting sqref="N5:N50">
     <cfRule type="expression" dxfId="3" priority="4">
       <formula>N5="در انتظار"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S5:S44">
+  <conditionalFormatting sqref="S5:S50">
     <cfRule type="expression" dxfId="0" priority="5">
       <formula>S5="تأیید شد"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S5:S44">
+  <conditionalFormatting sqref="S5:S50">
     <cfRule type="expression" dxfId="1" priority="6">
       <formula>S5="تأیید نشد"</formula>
     </cfRule>

</xml_diff>